<commit_message>
Refactor project monitoring and demo generation workflows
</commit_message>
<xml_diff>
--- a/V1.0需求（2026.6.11）/官方数据/中国产业链分类.xlsx
+++ b/V1.0需求（2026.6.11）/官方数据/中国产业链分类.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产业链-产业" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产业链汇总统计" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据来源说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产业链-产业" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产业链汇总统计" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'产业链-产业'!$A$1:$D$2054</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'产业链-产业'!$A$1:$D$2054</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +34,37 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="001F1F1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -65,8 +95,33 @@
         <bgColor rgb="00DAEEF3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7FBFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B9BD5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -80,11 +135,25 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -102,6 +171,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,6 +553,237 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>数据来源说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>工作簿</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>中国产业链分类.xlsx</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="10" t="n"/>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>说明生成日期</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>说明口径</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>本页汇总当前工作簿内可确认的数据来源、来源位置和使用边界；未在原文件中保存页面级来源的，已明确标注为待补源。</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>适用范围</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>本说明仅解释本工作簿数据来源，不改变后续数据 sheet 的原始内容。</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>来源类型</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>来源名称/文件</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>发布机构/网站</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>来源链接或本文件位置</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>覆盖数据范围</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>使用方式</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>可信度与边界说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="68" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>原始产业链分类表</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>中国产业链、产业、上中下游、代表企业整理表</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>本项目/公开资料二次整理</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>本文件未保存原始来源字段、隐藏来源表、批注或可追溯链接</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>产业链-产业、产业链汇总统计</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>作为产业链分类和代表企业基础表使用。</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>不能直接称为官方原表；上中下游和代表企业字段属于二次整理口径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="68" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>同目录补充研判</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>中国产业链分类-补充来源研判.xlsx</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>本项目整理</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>同目录文件：中国产业链分类-补充来源研判.xlsx</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>来源类型、建议引用来源、可信度、来源说明</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>为本表补充来源类型判断和官方口径参考。</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>后续若用于正式产品入库，仍需补充每条产业链的具体政策、研报、地方产业链图谱或企业公开资料页面。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>引用提示：用于汇报或正式材料时，优先引用本页中已列明的主管部门/官方网站链接；对“二次整理”“平台接口导出”“未保存原始 URL”的数据，应补充原始下载记录或页面级证据后再作为正式来源。</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B6:G6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -43646,7 +43966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>